<commit_message>
Orientar la app al público general y corregir la exportación a PDF
- Retirar las menciones a contenido docente, semana 4 y ejercicio de clase (app, README y plantilla Excel)
- PDF: sin cortes a la derecha en tablas, diagrama y calculadora; sin páginas casi vacías
- Quitar el «(opcional)» duplicado en la calculadora y usar signos de interrogación en la conclusión

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/plantilla_costo_punto_adherencia.xlsx
+++ b/downloads/plantilla_costo_punto_adherencia.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Ejercicio de clase · incentivo (ilustrativo)</t>
+          <t>Ejercicio ilustrativo · incentivo</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -983,12 +983,12 @@
     <row r="3" ht="75" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Ejercicio de clase</t>
+          <t>Ejercicio ilustrativo</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Datos ficticios con fines didácticos: incentivo de 240.000 pesos por paciente durante seis meses; adherencia del 50 % al 62 %, y del 52 % tras retirar el incentivo.</t>
+          <t>Datos ficticios: incentivo de 240.000 pesos por paciente durante seis meses; adherencia del 50 % al 62 %, y del 52 % tras retirar el incentivo.</t>
         </is>
       </c>
     </row>

</xml_diff>